<commit_message>
LSM6DSOX SPI test code
</commit_message>
<xml_diff>
--- a/piese.xlsx
+++ b/piese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Desktop\projects\micromouse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE626AE7-DC31-428C-827E-9D6B3DCBCBE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9833912-2255-4F80-A59F-D1B9FE894FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FFDE713F-859F-4B3F-BED4-C08AC22FA580}"/>
   </bookViews>
@@ -380,12 +380,6 @@
     <t>AP62300Z6-7 Diodes Incorporated | Voltage Regulators - DC DC Switching Regulators | DigiKey</t>
   </si>
   <si>
-    <t>NRS5040T3R3NMGJ</t>
-  </si>
-  <si>
-    <t>Taiyo Yuden</t>
-  </si>
-  <si>
     <t>NRS5040T3R3NMGJ Taiyo Yuden | Fixed Inductors | DigiKey</t>
   </si>
   <si>
@@ -461,9 +455,6 @@
     <t>AP62300Z6-7 | Voltage Regulators - DC DC Switching Regulators | DIODES | LCSC</t>
   </si>
   <si>
-    <t>NRS5040T3R3NMGJ | Fixed Inductors | Taiyo Yuden | LCSC</t>
-  </si>
-  <si>
     <t>TLV75533PDBVR | Voltage Regulators - Linear, Low Drop Out (LDO) Regulators | TI | LCSC</t>
   </si>
   <si>
@@ -510,6 +501,15 @@
   </si>
   <si>
     <t>RF-W7SP30TS-A44 REFOND - LED | RGB; SMD; PLCC6; 1,8÷2,4/2,7÷3,4/2,7÷3,4VDC; 3,5x2,8x1,8mm | Transfer Multisort Elektronik România</t>
+  </si>
+  <si>
+    <t>APV APH0420T3R3M</t>
+  </si>
+  <si>
+    <t>APV</t>
+  </si>
+  <si>
+    <t>APH0420T3R3M | Fixed Inductors | APV | LCSC</t>
   </si>
 </sst>
 </file>
@@ -648,7 +648,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CCF854A4-5F3D-4236-9B97-F4C57F0E67B7}" name="Table1" displayName="Table1" ref="A1:N24" totalsRowShown="0" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:N24" xr:uid="{CCF854A4-5F3D-4236-9B97-F4C57F0E67B7}"/>
+  <autoFilter ref="A1:N24" xr:uid="{CCF854A4-5F3D-4236-9B97-F4C57F0E67B7}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="LCSC"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N24">
     <sortCondition descending="1" ref="D1:D24"/>
   </sortState>
@@ -1026,16 +1032,16 @@
         <v>93</v>
       </c>
       <c r="L1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="M1" t="s">
         <v>94</v>
       </c>
       <c r="N1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" hidden="1">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1046,7 +1052,7 @@
         <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1078,7 +1084,7 @@
       </c>
       <c r="O2" s="9"/>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" hidden="1">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1086,10 +1092,10 @@
         <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1120,18 +1126,18 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" hidden="1">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C4" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E4">
         <v>10</v>
@@ -1162,18 +1168,18 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" hidden="1">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E5">
         <v>5</v>
@@ -1198,22 +1204,22 @@
         <v>0</v>
       </c>
       <c r="M5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="N5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" hidden="1">
       <c r="A6">
         <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -1238,7 +1244,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" hidden="1">
       <c r="A7">
         <v>19</v>
       </c>
@@ -1246,7 +1252,7 @@
         <v>77</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E7">
         <v>10</v>
@@ -1271,7 +1277,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" hidden="1">
       <c r="A8">
         <v>20</v>
       </c>
@@ -1279,7 +1285,7 @@
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E8">
         <v>10</v>
@@ -1305,15 +1311,15 @@
       </c>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" hidden="1">
       <c r="A9">
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -1335,18 +1341,18 @@
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" hidden="1">
       <c r="A10">
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -1376,13 +1382,13 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C11" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E11">
         <v>4</v>
@@ -1408,7 +1414,7 @@
         <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1416,13 +1422,13 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -1448,10 +1454,10 @@
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="N12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1459,13 +1465,13 @@
         <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C13" t="s">
         <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -1491,10 +1497,10 @@
         <v>0</v>
       </c>
       <c r="M13" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="N13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -1508,7 +1514,7 @@
         <v>96</v>
       </c>
       <c r="D14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -1534,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="N14" t="s">
         <v>100</v>
@@ -1551,7 +1557,7 @@
         <v>96</v>
       </c>
       <c r="D15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -1577,7 +1583,7 @@
         <v>0</v>
       </c>
       <c r="M15" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="N15" t="s">
         <v>103</v>
@@ -1594,7 +1600,7 @@
         <v>107</v>
       </c>
       <c r="D16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -1620,7 +1626,7 @@
         <v>0</v>
       </c>
       <c r="M16" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="N16" t="s">
         <v>108</v>
@@ -1637,7 +1643,7 @@
         <v>107</v>
       </c>
       <c r="D17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E17">
         <v>10</v>
@@ -1663,7 +1669,7 @@
         <v>0</v>
       </c>
       <c r="M17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="N17" t="s">
         <v>109</v>
@@ -1680,7 +1686,7 @@
         <v>110</v>
       </c>
       <c r="D18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -1706,7 +1712,7 @@
         <v>0</v>
       </c>
       <c r="M18" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="N18" t="s">
         <v>111</v>
@@ -1723,7 +1729,7 @@
         <v>112</v>
       </c>
       <c r="D19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E19">
         <v>50</v>
@@ -1749,7 +1755,7 @@
         <v>0</v>
       </c>
       <c r="M19" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="N19" t="s">
         <v>113</v>
@@ -1766,7 +1772,7 @@
         <v>115</v>
       </c>
       <c r="D20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -1792,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="M20" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="N20" t="s">
         <v>116</v>
@@ -1803,27 +1809,27 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="C21" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D21" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E21">
         <v>10</v>
       </c>
       <c r="F21">
-        <v>0.85</v>
+        <v>0.42</v>
       </c>
       <c r="G21">
         <f t="shared" si="1"/>
-        <v>1.0285</v>
+        <v>0.50819999999999999</v>
       </c>
       <c r="H21">
         <f t="shared" si="0"/>
-        <v>10.285</v>
+        <v>5.0819999999999999</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -1834,11 +1840,11 @@
       <c r="L21">
         <v>0</v>
       </c>
-      <c r="M21" t="s">
-        <v>144</v>
+      <c r="M21" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="N21" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -1852,7 +1858,7 @@
         <v>110</v>
       </c>
       <c r="D22" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E22">
         <v>10</v>
@@ -1878,10 +1884,10 @@
         <v>0</v>
       </c>
       <c r="M22" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="N22" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -1889,13 +1895,13 @@
         <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E23">
         <v>20</v>
@@ -1921,15 +1927,15 @@
         <v>0</v>
       </c>
       <c r="M23" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" hidden="1">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G24">
         <f t="shared" si="1"/>
@@ -1946,7 +1952,7 @@
         <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -1963,13 +1969,16 @@
     <row r="27" spans="1:14">
       <c r="B27" s="7">
         <f>SUM(Table1[Total Price])</f>
-        <v>636.50389999999993</v>
+        <v>631.30089999999996</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
     </row>
     <row r="28" spans="1:14">
-      <c r="G28" s="8"/>
+      <c r="G28" s="8">
+        <f>SUM(H11:H23)</f>
+        <v>243.56089999999998</v>
+      </c>
       <c r="H28" s="8"/>
     </row>
   </sheetData>
@@ -2004,16 +2013,16 @@
     <hyperlink ref="M18" r:id="rId25" display="https://www.lcsc.com/product-detail/C398355.html?s_z=n_q_x_TLV9062IDR&amp;spm=wm.ssy.em.0.tz&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbVF1RRVZYVjsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktXRVddSQwSGg0%3D" xr:uid="{0EC453CE-6CE2-4B90-A97C-94128C5CD7D8}"/>
     <hyperlink ref="M19" r:id="rId26" display="https://www.lcsc.com/product-detail/C20917.html?s_z=n_q_AO3400A&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1RSQVNeUDsOAxUeFF5JWBYZEEoKFBINSQcJGk4dAgUUFAk%3D" xr:uid="{CC1EEA12-849E-4A66-8EC8-104A221385AC}"/>
     <hyperlink ref="M20" r:id="rId27" display="https://www.lcsc.com/product-detail/C5250745.html?s_z=n_q_AP62300Z6-7&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1VTQ1lXVjsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktXRlRbSQwSGg0%3D" xr:uid="{12149DD9-B80B-4EB6-8FD1-A461639AFB0E}"/>
-    <hyperlink ref="M21" r:id="rId28" display="https://www.lcsc.com/product-detail/C222946.html?s_z=n_q_NRS5040T3R3NMGJ&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1ZVRFZeXzsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaSgADAwAHC0slQlNbV1NSQk8GEwkK" xr:uid="{97471ABE-2B04-4FC5-9C07-60239F786D72}"/>
-    <hyperlink ref="M22" r:id="rId29" display="https://www.lcsc.com/product-detail/C404027.html?s_z=n_q_TLV75533PDBVR&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1dWQVRcUjsOAxUeFF5JWBYZEEoKFBINSQcJGk4dAgUUFAk%3D" xr:uid="{08C2F20C-33D4-436E-B599-6C93FCF6DD96}"/>
-    <hyperlink ref="M12" r:id="rId30" display="https://www.lcsc.com/product-detail/C141517.html?s_z=n_q_TB6612FNG&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1dQTlBeXjsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktXRVZeSQwSGg0%3D" xr:uid="{13F8DA37-370F-4375-855D-D5CE1AEF859B}"/>
-    <hyperlink ref="M13" r:id="rId31" display="https://www.lcsc.com/product-detail/C118301.html?s_z=n_q_TEFT4300&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1BTRFJYUzsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktXQ1VfSQwSGg0%3D" xr:uid="{300A3969-0246-4367-9525-EE759EDAA06E}"/>
-    <hyperlink ref="M11" r:id="rId32" display="https://www.lcsc.com/product-detail/C50203010.html?s_z=n_q_MT6701CT-ACD&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVYUlJVT1JXVzsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaSgADAwAHC0slRFFeVFVfQU8GEwkK" xr:uid="{A65D1758-9698-480B-850A-E674A538086D}"/>
-    <hyperlink ref="M23" r:id="rId33" display="https://www.lcsc.com/product-detail/C19829543.html?s_z=n_q_ESD3V3U1U&amp;spm=wm.fly.bg.1.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVYUV1TT1heVTsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktRR1NADxALGw%3D%3D" xr:uid="{07BA1E9B-C7EC-4AA1-A9E3-5EC19B289B5B}"/>
-    <hyperlink ref="M2" r:id="rId34" display="https://www.tme.eu/ro/details/nucleo-f411re/kituri-de-dezvoltare-stm/stmicroelectronics/" xr:uid="{69170CFE-C5E3-48E5-93D2-791D489D990A}"/>
-    <hyperlink ref="M3" r:id="rId35" display="https://www.tme.eu/ro/details/abx00101/solutii-arduino/arduino/modulino-movement/" xr:uid="{F144BF92-4ED3-4998-AFDE-91611CE0E743}"/>
-    <hyperlink ref="M4" r:id="rId36" display="https://www.tme.eu/ro/details/8.00m-smdhc49s/resonators-and-generators/yic/" xr:uid="{220F2AB7-0894-4030-8B00-577AB6BCB560}"/>
-    <hyperlink ref="M5" r:id="rId37" display="https://www.tme.eu/ro/details/rf-w7sp30ts-a44/diode-led-smd-colorate/refond/" xr:uid="{EE57C078-EEE4-4A22-914E-A167F898EF55}"/>
+    <hyperlink ref="M22" r:id="rId28" display="https://www.lcsc.com/product-detail/C404027.html?s_z=n_q_TLV75533PDBVR&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1dWQVRcUjsOAxUeFF5JWBYZEEoKFBINSQcJGk4dAgUUFAk%3D" xr:uid="{08C2F20C-33D4-436E-B599-6C93FCF6DD96}"/>
+    <hyperlink ref="M12" r:id="rId29" display="https://www.lcsc.com/product-detail/C141517.html?s_z=n_q_TB6612FNG&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1dQTlBeXjsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktXRVZeSQwSGg0%3D" xr:uid="{13F8DA37-370F-4375-855D-D5CE1AEF859B}"/>
+    <hyperlink ref="M13" r:id="rId30" display="https://www.lcsc.com/product-detail/C118301.html?s_z=n_q_TEFT4300&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVbU1BTRFJYUzsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktXQ1VfSQwSGg0%3D" xr:uid="{300A3969-0246-4367-9525-EE759EDAA06E}"/>
+    <hyperlink ref="M11" r:id="rId31" display="https://www.lcsc.com/product-detail/C50203010.html?s_z=n_q_MT6701CT-ACD&amp;spm=wm.fly.bg.0.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVYUlJVT1JXVzsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaSgADAwAHC0slRFFeVFVfQU8GEwkK" xr:uid="{A65D1758-9698-480B-850A-E674A538086D}"/>
+    <hyperlink ref="M23" r:id="rId32" display="https://www.lcsc.com/product-detail/C19829543.html?s_z=n_q_ESD3V3U1U&amp;spm=wm.fly.bg.1.xh&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVVYUV1TT1heVTsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktRR1NADxALGw%3D%3D" xr:uid="{07BA1E9B-C7EC-4AA1-A9E3-5EC19B289B5B}"/>
+    <hyperlink ref="M2" r:id="rId33" display="https://www.tme.eu/ro/details/nucleo-f411re/kituri-de-dezvoltare-stm/stmicroelectronics/" xr:uid="{69170CFE-C5E3-48E5-93D2-791D489D990A}"/>
+    <hyperlink ref="M3" r:id="rId34" display="https://www.tme.eu/ro/details/abx00101/solutii-arduino/arduino/modulino-movement/" xr:uid="{F144BF92-4ED3-4998-AFDE-91611CE0E743}"/>
+    <hyperlink ref="M4" r:id="rId35" display="https://www.tme.eu/ro/details/8.00m-smdhc49s/resonators-and-generators/yic/" xr:uid="{220F2AB7-0894-4030-8B00-577AB6BCB560}"/>
+    <hyperlink ref="M5" r:id="rId36" display="https://www.tme.eu/ro/details/rf-w7sp30ts-a44/diode-led-smd-colorate/refond/" xr:uid="{EE57C078-EEE4-4A22-914E-A167F898EF55}"/>
+    <hyperlink ref="M21" r:id="rId37" display="https://www.lcsc.com/product-detail/C5349667.html?s_z=n_q_t_3.3uH&amp;spm=wm.fly.bg.7.xh___wm.ssy.tc.0.tz&amp;lcsc_vid=FQBfBVRVQAUPVVdQFlIPBFJeQQcNVF1XRQINUgFWFVAxVlNeQVRbUF1QRFBcVjsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaSgADAwAHC0slRVNcXlBQWQkaCgg%3D" xr:uid="{8B513A70-CC11-46C3-9112-7E18CAB3040F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
PCB proj + components import in lib
</commit_message>
<xml_diff>
--- a/piese.xlsx
+++ b/piese.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Desktop\projects\micromouse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9833912-2255-4F80-A59F-D1B9FE894FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D2E965-468B-4F7E-9798-8B86A0F0E30C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FFDE713F-859F-4B3F-BED4-C08AC22FA580}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FFDE713F-859F-4B3F-BED4-C08AC22FA580}"/>
   </bookViews>
   <sheets>
     <sheet name="parts" sheetId="5" r:id="rId1"/>
@@ -648,13 +648,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CCF854A4-5F3D-4236-9B97-F4C57F0E67B7}" name="Table1" displayName="Table1" ref="A1:N24" totalsRowShown="0" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:N24" xr:uid="{CCF854A4-5F3D-4236-9B97-F4C57F0E67B7}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="LCSC"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:N24" xr:uid="{CCF854A4-5F3D-4236-9B97-F4C57F0E67B7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N24">
     <sortCondition descending="1" ref="D1:D24"/>
   </sortState>
@@ -1041,7 +1035,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:15" hidden="1">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1084,7 +1078,7 @@
       </c>
       <c r="O2" s="9"/>
     </row>
-    <row r="3" spans="1:15" hidden="1">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1126,7 +1120,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:15" hidden="1">
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1168,7 +1162,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:15" hidden="1">
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1211,7 +1205,7 @@
       </c>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" spans="1:15" hidden="1">
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>18</v>
       </c>
@@ -1244,7 +1238,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:15" hidden="1">
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>19</v>
       </c>
@@ -1277,7 +1271,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:15" hidden="1">
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>20</v>
       </c>
@@ -1311,7 +1305,7 @@
       </c>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="1:15" hidden="1">
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>21</v>
       </c>
@@ -1344,7 +1338,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:15" hidden="1">
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>22</v>
       </c>
@@ -1930,7 +1924,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="24" spans="1:14" hidden="1">
+    <row r="24" spans="1:14">
       <c r="A24">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
LCSC lib moved + uC minimal
</commit_message>
<xml_diff>
--- a/piese.xlsx
+++ b/piese.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Desktop\projects\micromouse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D2E965-468B-4F7E-9798-8B86A0F0E30C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66974AE-8914-48DB-808F-895401101CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FFDE713F-859F-4B3F-BED4-C08AC22FA580}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FFDE713F-859F-4B3F-BED4-C08AC22FA580}"/>
   </bookViews>
   <sheets>
     <sheet name="parts" sheetId="5" r:id="rId1"/>

</xml_diff>